<commit_message>
Add missing comments and few fixes
</commit_message>
<xml_diff>
--- a/data/20230131_Curve.xlsx
+++ b/data/20230131_Curve.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utente\Documents\A_Documenti\Roberto Documents\A_Politecnico\Corsi\FinancialEngineering\ProgettiFinali\2023\Project_1_SwapWithCVA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10739941_polimi_it/Documents/GITHUB/Amortizing-Swap-Pricing-with-CVA-under-a-Multi-Curve-Framework/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D42CED78-C2D2-4EA1-9469-C3520212724A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{D42CED78-C2D2-4EA1-9469-C3520212724A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9C70AF0-D4FF-5080-9E75-583621377A43}"/>
   <bookViews>
-    <workbookView xWindow="1812" yWindow="3000" windowWidth="18468" windowHeight="10680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1073" yWindow="842" windowWidth="19562" windowHeight="10162" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Curve 3M 31 Jan" sheetId="2" r:id="rId1"/>
@@ -730,9 +730,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema di Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -770,9 +770,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -805,26 +805,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -857,26 +840,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1051,12 +1017,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="6" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="6" width="9.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1076,7 +1042,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1096,7 +1062,7 @@
         <v>0.99382800000000004</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1116,7 +1082,7 @@
         <v>0.99238599999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1136,7 +1102,7 @@
         <v>0.98918200000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1156,7 +1122,7 @@
         <v>0.98678500000000002</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -1176,7 +1142,7 @@
         <v>0.98406800000000005</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -1196,7 +1162,7 @@
         <v>0.98063500000000003</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -1216,7 +1182,7 @@
         <v>0.97816099999999995</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -1236,7 +1202,7 @@
         <v>0.97203200000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -1256,7 +1222,7 @@
         <v>0.93866000000000005</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -1276,7 +1242,7 @@
         <v>0.91435999999999995</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1296,7 +1262,7 @@
         <v>0.89132599999999995</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -1316,7 +1282,7 @@
         <v>0.86854100000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -1336,7 +1302,7 @@
         <v>0.84601199999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1356,7 +1322,7 @@
         <v>0.82345000000000002</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -1376,7 +1342,7 @@
         <v>0.80080700000000005</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1396,7 +1362,7 @@
         <v>0.77798800000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -1416,7 +1382,7 @@
         <v>0.75494700000000003</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -1436,7 +1402,7 @@
         <v>0.73238199999999998</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -1456,7 +1422,7 @@
         <v>0.71068299999999995</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -1476,7 +1442,7 @@
         <v>0.652397</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -1496,7 +1462,7 @@
         <v>0.58329900000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -1516,7 +1482,7 @@
         <v>0.53676000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -1536,7 +1502,7 @@
         <v>0.50012299999999998</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -1556,7 +1522,7 @@
         <v>0.44049199999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -1584,12 +1550,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="6" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="6" width="9.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1609,7 +1575,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -1629,7 +1595,7 @@
         <v>0.99961599999999995</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1649,7 +1615,7 @@
         <v>0.99914800000000004</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -1669,7 +1635,7 @@
         <v>0.99821400000000005</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -1689,7 +1655,7 @@
         <v>0.99593500000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1709,7 +1675,7 @@
         <v>0.99365199999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -1729,7 +1695,7 @@
         <v>0.99102800000000002</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -1749,7 +1715,7 @@
         <v>0.98828499999999997</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -1769,7 +1735,7 @@
         <v>0.98554399999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>38</v>
       </c>
@@ -1789,7 +1755,7 @@
         <v>0.98247200000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -1809,7 +1775,7 @@
         <v>0.97987500000000005</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -1829,7 +1795,7 @@
         <v>0.97701000000000005</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>41</v>
       </c>
@@ -1849,7 +1815,7 @@
         <v>0.97409500000000004</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>42</v>
       </c>
@@ -1869,7 +1835,7 @@
         <v>0.97147300000000003</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -1889,7 +1855,7 @@
         <v>0.96869400000000006</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>44</v>
       </c>
@@ -1909,7 +1875,7 @@
         <v>0.953681</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -1929,7 +1895,7 @@
         <v>0.94053799999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>15</v>
       </c>
@@ -1949,7 +1915,7 @@
         <v>0.91778899999999997</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -1969,7 +1935,7 @@
         <v>0.89642999999999995</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1989,7 +1955,7 @@
         <v>0.87549999999999994</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -2009,7 +1975,7 @@
         <v>0.85477300000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -2029,7 +1995,7 @@
         <v>0.83402699999999996</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>20</v>
       </c>
@@ -2049,7 +2015,7 @@
         <v>0.81319399999999997</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -2069,7 +2035,7 @@
         <v>0.79203599999999996</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -2089,7 +2055,7 @@
         <v>0.77046300000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -2109,7 +2075,7 @@
         <v>0.74931300000000001</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>24</v>
       </c>
@@ -2129,7 +2095,7 @@
         <v>0.72856100000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>25</v>
       </c>
@@ -2149,7 +2115,7 @@
         <v>0.67245999999999995</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>26</v>
       </c>
@@ -2169,7 +2135,7 @@
         <v>0.60410399999999997</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>27</v>
       </c>
@@ -2189,7 +2155,7 @@
         <v>0.55641499999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>28</v>
       </c>
@@ -2209,7 +2175,7 @@
         <v>0.51695400000000002</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>29</v>
       </c>
@@ -2229,7 +2195,7 @@
         <v>0.45313500000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>30</v>
       </c>

</xml_diff>